<commit_message>
CFA considering alternative models: 4-Factor Model A (Visualization Clarity + Visualization Retrieval) + Cognitive + Intuitiveness 4-Factor Model B (Visualization - 'trialError') + (Cognitive - 'taskComplete'), +new factor (trialError + taskComplete) + Intuitiveness 3-Factor Model A: Our selection of Visualization + Cognitive + Intuitiveness) 3-Factor Model B: Our selection of items without trialError item 3-Factor Model C: Our selection of items without taskCompletion item 3-Factor Model D: Our selection of items without trialError and taskCompletion items 2-Factor Model A: Interface Usability vs. Cognitive Utility 2-Factor Model B (Alternative: System Experience vs. Intuitiveness) 1-Factor Model: Unidimensional Structure with all items
</commit_message>
<xml_diff>
--- a/Reproduce6 - AnalysisBySystem/Data_Analysis/generatedData/CFA_Model_Fit_Comparison.xlsx
+++ b/Reproduce6 - AnalysisBySystem/Data_Analysis/generatedData/CFA_Model_Fit_Comparison.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
   <si>
     <t xml:space="preserve">Model</t>
   </si>
@@ -61,10 +61,22 @@
     <t xml:space="preserve">Pooled_2_Factor_B</t>
   </si>
   <si>
-    <t xml:space="preserve">Pooled_3_Factor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pooled_4_Factor</t>
+    <t xml:space="preserve">Pooled_3_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pooled_3_Factor_B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pooled_3_Factor_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pooled_3_Factor_D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pooled_4_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pooled_4_Factor_B</t>
   </si>
   <si>
     <t xml:space="preserve">Multigroup_1_Factor</t>
@@ -76,10 +88,22 @@
     <t xml:space="preserve">Multigroup_2_Factor_B</t>
   </si>
   <si>
-    <t xml:space="preserve">Multigroup_3_Factor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multigroup_4_Factor</t>
+    <t xml:space="preserve">Multigroup_3_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multigroup_3_Factor_B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multigroup_3_Factor_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multigroup_3_Factor_D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multigroup_4_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multigroup_4_Factor_B</t>
   </si>
   <si>
     <t xml:space="preserve">Tableau_1_Factor</t>
@@ -91,10 +115,22 @@
     <t xml:space="preserve">Tableau_2_Factor_B</t>
   </si>
   <si>
-    <t xml:space="preserve">Tableau_3_Factor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tableau_4_Factor</t>
+    <t xml:space="preserve">Tableau_3_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tableau_3_Factor_B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tableau_3_Factor_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tableau_3_Factor_D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tableau_4_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tableau_4_Factor_B</t>
   </si>
   <si>
     <t xml:space="preserve">JMP_1_Factor</t>
@@ -106,10 +142,22 @@
     <t xml:space="preserve">JMP_2_Factor_B</t>
   </si>
   <si>
-    <t xml:space="preserve">JMP_3_Factor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JMP_4_Factor</t>
+    <t xml:space="preserve">JMP_3_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JMP_3_Factor_B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JMP_3_Factor_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JMP_3_Factor_D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JMP_4_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JMP_4_Factor_B</t>
   </si>
   <si>
     <t xml:space="preserve">Excel_1_Factor</t>
@@ -121,10 +169,22 @@
     <t xml:space="preserve">Excel_2_Factor_B</t>
   </si>
   <si>
-    <t xml:space="preserve">Excel_3_Factor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Excel_4_Factor</t>
+    <t xml:space="preserve">Excel_3_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excel_3_Factor_B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excel_3_Factor_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excel_3_Factor_D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excel_4_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excel_4_Factor_B</t>
   </si>
   <si>
     <t xml:space="preserve">Data Studio_1_Factor</t>
@@ -136,10 +196,22 @@
     <t xml:space="preserve">Data Studio_2_Factor_B</t>
   </si>
   <si>
-    <t xml:space="preserve">Data Studio_3_Factor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data Studio_4_Factor</t>
+    <t xml:space="preserve">Data Studio_3_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Studio_3_Factor_B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Studio_3_Factor_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Studio_3_Factor_D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Studio_4_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Studio_4_Factor_B</t>
   </si>
   <si>
     <t xml:space="preserve">Power BI_1_Factor</t>
@@ -151,10 +223,22 @@
     <t xml:space="preserve">Power BI_2_Factor_B</t>
   </si>
   <si>
-    <t xml:space="preserve">Power BI_3_Factor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Power BI_4_Factor</t>
+    <t xml:space="preserve">Power BI_3_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power BI_3_Factor_B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power BI_3_Factor_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power BI_3_Factor_D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power BI_4_Factor_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power BI_4_Factor_B</t>
   </si>
 </sst>
 </file>
@@ -678,37 +762,189 @@
         <v>16</v>
       </c>
       <c r="B6" t="n">
+        <v>150.306302605196</v>
+      </c>
+      <c r="C6" t="n">
+        <v>51</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.0000000000100007779835209</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.899517953942614</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.869964410984559</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.0928216103352906</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.075848481008825</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.110188225940055</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.0623331237103484</v>
+      </c>
+      <c r="K6" t="n">
+        <v>6104.36541664442</v>
+      </c>
+      <c r="L6" t="n">
+        <v>6237.76628161604</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="n">
+        <v>138.591975254452</v>
+      </c>
+      <c r="C7" t="n">
+        <v>51</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.000000000498310503971311</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.907778565608746</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.8806546143172</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.0871751799252927</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.0699342268035676</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.104752114981732</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.0601704124169632</v>
+      </c>
+      <c r="K7" t="n">
+        <v>6262.98987097161</v>
+      </c>
+      <c r="L7" t="n">
+        <v>6396.39073594323</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="n">
+        <v>121.34055633536</v>
+      </c>
+      <c r="C8" t="n">
+        <v>41</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.00000000070812211649951</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.908533722539004</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.877301335113297</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.0931153477334798</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.0742260986550067</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.112496889154063</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.062140249672347</v>
+      </c>
+      <c r="K8" t="n">
+        <v>5663.88628942492</v>
+      </c>
+      <c r="L8" t="n">
+        <v>5787.02554939872</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="n">
         <v>167.593454540538</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C9" t="n">
         <v>59</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D9" t="n">
         <v>0.00000000000241406894474494</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E9" t="n">
         <v>0.897546353411808</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F9" t="n">
         <v>0.864552806205441</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G9" t="n">
         <v>0.0902446778787873</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H9" t="n">
         <v>0.0743444940660238</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I9" t="n">
         <v>0.106465022032753</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J9" t="n">
         <v>0.0603781110003134</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K9" t="n">
         <v>6708.31406168231</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L9" t="n">
         <v>6862.23813664956</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="n">
+        <v>157.411274189354</v>
+      </c>
+      <c r="C10" t="n">
+        <v>59</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.0000000000679075684573149</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.907152839471316</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.877252906419705</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.0859096999201751</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.0698068233446634</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.102289204992074</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.0586676869317133</v>
+      </c>
+      <c r="K10" t="n">
+        <v>6698.13188133112</v>
+      </c>
+      <c r="L10" t="n">
+        <v>6852.05595629838</v>
       </c>
     </row>
   </sheetData>
@@ -762,7 +998,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B2" t="n">
         <v>701.66679519203</v>
@@ -800,7 +1036,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B3" t="n">
         <v>664.304887503506</v>
@@ -838,7 +1074,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B4" t="n">
         <v>554.976322683786</v>
@@ -876,7 +1112,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B5" t="n">
         <v>511.372951817928</v>
@@ -914,40 +1150,192 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B6" t="n">
+        <v>420.293251093961</v>
+      </c>
+      <c r="C6" t="n">
+        <v>255</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.000000000315974135745023</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.842456478156931</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.796120148203087</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.12482765309189</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.103172948827158</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.145822928725743</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.10404675331768</v>
+      </c>
+      <c r="K6" t="n">
+        <v>5640.46568478349</v>
+      </c>
+      <c r="L6" t="n">
+        <v>6291.28561032525</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="n">
+        <v>403.29274173874</v>
+      </c>
+      <c r="C7" t="n">
+        <v>255</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.00000000890872964287581</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.855668539989919</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.813218110575189</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.118234220332881</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.095915627341797</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.139666802279768</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.0997330823098637</v>
+      </c>
+      <c r="K7" t="n">
+        <v>5757.859117777</v>
+      </c>
+      <c r="L7" t="n">
+        <v>6408.67904331875</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="n">
+        <v>323.383810407694</v>
+      </c>
+      <c r="C8" t="n">
+        <v>205</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.000000251139192664063</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.871655240748164</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.827830201003634</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.117820961182467</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.0927856678755091</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.141721283322549</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.0995979153025139</v>
+      </c>
+      <c r="K8" t="n">
+        <v>5222.46766588282</v>
+      </c>
+      <c r="L8" t="n">
+        <v>5823.22452022906</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="n">
         <v>488.183934833955</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C9" t="n">
         <v>295</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D9" t="n">
         <v>0.0000000000101690877940541</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E9" t="n">
         <v>0.832816356964875</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F9" t="n">
         <v>0.778977556665428</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G9" t="n">
         <v>0.125466513695207</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H9" t="n">
         <v>0.105419156585376</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I9" t="n">
         <v>0.144963287827565</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J9" t="n">
         <v>0.100537111305942</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K9" t="n">
         <v>6187.56717394689</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L9" t="n">
         <v>6938.51324187969</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" t="n">
+        <v>476.753996823711</v>
+      </c>
+      <c r="C10" t="n">
+        <v>295</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.0000000000993222171175034</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.842707959379231</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.792054590365763</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.121698243961934</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.101322271134089</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.141421249861777</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.0993071542207653</v>
+      </c>
+      <c r="K10" t="n">
+        <v>6176.13723593665</v>
+      </c>
+      <c r="L10" t="n">
+        <v>6927.08330386944</v>
       </c>
     </row>
   </sheetData>
@@ -1001,7 +1389,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="B2" t="n">
         <v>107.628820962087</v>
@@ -1039,7 +1427,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B3" t="n">
         <v>99.4005152315861</v>
@@ -1077,7 +1465,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B4" t="n">
         <v>96.407481982889</v>
@@ -1115,7 +1503,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="B5" t="n">
         <v>89.4364571191219</v>
@@ -1153,800 +1541,1560 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B6" t="n">
-        <v>85.0683931693357</v>
+        <v>74.6957984715062</v>
       </c>
       <c r="C6" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01478340643864</v>
+        <v>0.016936963830653</v>
       </c>
       <c r="E6" t="n">
-        <v>0.843966297241303</v>
+        <v>0.848512451673682</v>
       </c>
       <c r="F6" t="n">
-        <v>0.793718155674943</v>
+        <v>0.803957290401236</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0980058973781927</v>
+        <v>0.100501297789728</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0448849229582346</v>
+        <v>0.0439425542224866</v>
       </c>
       <c r="I6" t="n">
-        <v>0.141927880560955</v>
+        <v>0.147219138819872</v>
       </c>
       <c r="J6" t="n">
-        <v>0.107800550239472</v>
+        <v>0.112802186167895</v>
       </c>
       <c r="K6" t="n">
-        <v>1435.55975624985</v>
+        <v>1297.31019066572</v>
       </c>
       <c r="L6" t="n">
-        <v>1517.84861909186</v>
+        <v>1368.62720512879</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B7" t="n">
-        <v>150.484617896652</v>
+        <v>63.2275160659504</v>
       </c>
       <c r="C7" t="n">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="D7" t="n">
-        <v>0.00000000986938220037814</v>
+        <v>0.116941784649122</v>
       </c>
       <c r="E7" t="n">
-        <v>0.659403098980474</v>
+        <v>0.917788457032285</v>
       </c>
       <c r="F7" t="n">
-        <v>0.591283718776568</v>
+        <v>0.893608591453545</v>
       </c>
       <c r="G7" t="n">
-        <v>0.179099915406334</v>
+        <v>0.0721946669383218</v>
       </c>
       <c r="H7" t="n">
-        <v>0.141749038418387</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0.216696219423615</v>
+        <v>0.124898278522399</v>
       </c>
       <c r="J7" t="n">
-        <v>0.120321995249397</v>
+        <v>0.094361365876153</v>
       </c>
       <c r="K7" t="n">
-        <v>1228.01508629812</v>
+        <v>1331.56537154558</v>
       </c>
       <c r="L7" t="n">
-        <v>1294.84439689959</v>
+        <v>1402.88238600866</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B8" t="n">
-        <v>150.453650133903</v>
+        <v>50.850857654777</v>
       </c>
       <c r="C8" t="n">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="D8" t="n">
-        <v>0.00000000640108632765646</v>
+        <v>0.139283761761149</v>
       </c>
       <c r="E8" t="n">
-        <v>0.65554217773971</v>
+        <v>0.929407117825334</v>
       </c>
       <c r="F8" t="n">
-        <v>0.580192029120271</v>
+        <v>0.905302231229107</v>
       </c>
       <c r="G8" t="n">
-        <v>0.181513843007825</v>
+        <v>0.0722713517191224</v>
       </c>
       <c r="H8" t="n">
-        <v>0.144041000995474</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>0.219285642762058</v>
+        <v>0.13055238283785</v>
       </c>
       <c r="J8" t="n">
-        <v>0.120283418091262</v>
+        <v>0.0941143100595579</v>
       </c>
       <c r="K8" t="n">
-        <v>1229.98411853538</v>
+        <v>1194.85123935255</v>
       </c>
       <c r="L8" t="n">
-        <v>1298.52700120355</v>
+        <v>1260.68232962615</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B9" t="n">
-        <v>144.613293690626</v>
+        <v>85.0683931693357</v>
       </c>
       <c r="C9" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0000000357300483644352</v>
+        <v>0.01478340643864</v>
       </c>
       <c r="E9" t="n">
-        <v>0.678811946668602</v>
+        <v>0.843966297241303</v>
       </c>
       <c r="F9" t="n">
-        <v>0.608552060002358</v>
+        <v>0.793718155674943</v>
       </c>
       <c r="G9" t="n">
-        <v>0.175275581892368</v>
+        <v>0.0980058973781927</v>
       </c>
       <c r="H9" t="n">
-        <v>0.137350962321125</v>
+        <v>0.0448849229582346</v>
       </c>
       <c r="I9" t="n">
-        <v>0.21336166603199</v>
+        <v>0.141927880560955</v>
       </c>
       <c r="J9" t="n">
-        <v>0.116508255091567</v>
+        <v>0.107800550239472</v>
       </c>
       <c r="K9" t="n">
-        <v>1224.1437620921</v>
+        <v>1435.55975624985</v>
       </c>
       <c r="L9" t="n">
-        <v>1292.68664476027</v>
+        <v>1517.84861909186</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="B10" t="n">
-        <v>137.136307313497</v>
+        <v>70.5151144799642</v>
       </c>
       <c r="C10" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D10" t="n">
-        <v>0.000000132783266604264</v>
+        <v>0.144915399509547</v>
       </c>
       <c r="E10" t="n">
-        <v>0.70063393795634</v>
+        <v>0.931075692378593</v>
       </c>
       <c r="F10" t="n">
-        <v>0.623378180009589</v>
+        <v>0.908879728907292</v>
       </c>
       <c r="G10" t="n">
-        <v>0.171924254763206</v>
+        <v>0.065137218350421</v>
       </c>
       <c r="H10" t="n">
-        <v>0.133120611372242</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>0.210804734654672</v>
+        <v>0.116388312659431</v>
       </c>
       <c r="J10" t="n">
-        <v>0.113027653260856</v>
+        <v>0.0915800484024921</v>
       </c>
       <c r="K10" t="n">
-        <v>1220.66677571497</v>
+        <v>1421.00647756048</v>
       </c>
       <c r="L10" t="n">
-        <v>1292.63680251655</v>
+        <v>1503.29534040249</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="B11" t="n">
-        <v>130.476919533878</v>
+        <v>150.484617896652</v>
       </c>
       <c r="C11" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="D11" t="n">
-        <v>0.000000255995186160263</v>
+        <v>0.00000000986938220037814</v>
       </c>
       <c r="E11" t="n">
-        <v>0.715214059714313</v>
+        <v>0.659403098980474</v>
       </c>
       <c r="F11" t="n">
-        <v>0.623503333181634</v>
+        <v>0.591283718776568</v>
       </c>
       <c r="G11" t="n">
-        <v>0.171895686777327</v>
+        <v>0.179099915406334</v>
       </c>
       <c r="H11" t="n">
-        <v>0.132111414779108</v>
+        <v>0.141749038418387</v>
       </c>
       <c r="I11" t="n">
-        <v>0.211757737314802</v>
+        <v>0.216696219423615</v>
       </c>
       <c r="J11" t="n">
-        <v>0.112319231522081</v>
+        <v>0.120321995249397</v>
       </c>
       <c r="K11" t="n">
-        <v>1220.00738793535</v>
+        <v>1228.01508629812</v>
       </c>
       <c r="L11" t="n">
-        <v>1297.11813093704</v>
+        <v>1294.84439689959</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="B12" t="n">
-        <v>125.400089023988</v>
+        <v>150.453650133903</v>
       </c>
       <c r="C12" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0000101966242739282</v>
+        <v>0.00000000640108632765646</v>
       </c>
       <c r="E12" t="n">
-        <v>0.662533424144711</v>
+        <v>0.65554217773971</v>
       </c>
       <c r="F12" t="n">
-        <v>0.595040108973653</v>
+        <v>0.580192029120271</v>
       </c>
       <c r="G12" t="n">
-        <v>0.165318955429887</v>
+        <v>0.181513843007825</v>
       </c>
       <c r="H12" t="n">
-        <v>0.121314349533521</v>
+        <v>0.144041000995474</v>
       </c>
       <c r="I12" t="n">
-        <v>0.208503860596322</v>
+        <v>0.219285642762058</v>
       </c>
       <c r="J12" t="n">
-        <v>0.105344773717229</v>
+        <v>0.120283418091262</v>
       </c>
       <c r="K12" t="n">
-        <v>1062.90684577687</v>
+        <v>1229.98411853538</v>
       </c>
       <c r="L12" t="n">
-        <v>1122.4349062369</v>
+        <v>1298.52700120355</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="B13" t="n">
-        <v>115.947271574653</v>
+        <v>144.613293690626</v>
       </c>
       <c r="C13" t="n">
         <v>64</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0000765350681616317</v>
+        <v>0.0000000357300483644352</v>
       </c>
       <c r="E13" t="n">
-        <v>0.709760893624499</v>
+        <v>0.678811946668602</v>
       </c>
       <c r="F13" t="n">
-        <v>0.646271089104858</v>
+        <v>0.608552060002358</v>
       </c>
       <c r="G13" t="n">
-        <v>0.154508339614438</v>
+        <v>0.175275581892368</v>
       </c>
       <c r="H13" t="n">
-        <v>0.108579584351779</v>
+        <v>0.137350962321125</v>
       </c>
       <c r="I13" t="n">
-        <v>0.198890851377964</v>
+        <v>0.21336166603199</v>
       </c>
       <c r="J13" t="n">
-        <v>0.100644712505223</v>
+        <v>0.116508255091567</v>
       </c>
       <c r="K13" t="n">
-        <v>1055.45402832754</v>
+        <v>1224.1437620921</v>
       </c>
       <c r="L13" t="n">
-        <v>1116.50844931218</v>
+        <v>1292.68664476027</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="B14" t="n">
-        <v>101.610076724027</v>
+        <v>137.136307313497</v>
       </c>
       <c r="C14" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D14" t="n">
-        <v>0.00192967430381552</v>
+        <v>0.000000132783266604264</v>
       </c>
       <c r="E14" t="n">
-        <v>0.789865478432134</v>
+        <v>0.70063393795634</v>
       </c>
       <c r="F14" t="n">
-        <v>0.743898551839163</v>
+        <v>0.623378180009589</v>
       </c>
       <c r="G14" t="n">
-        <v>0.131468789498287</v>
+        <v>0.171924254763206</v>
       </c>
       <c r="H14" t="n">
-        <v>0.0803594558335405</v>
+        <v>0.133120611372242</v>
       </c>
       <c r="I14" t="n">
-        <v>0.178190348491534</v>
+        <v>0.210804734654672</v>
       </c>
       <c r="J14" t="n">
-        <v>0.0968710022278117</v>
+        <v>0.113027653260856</v>
       </c>
       <c r="K14" t="n">
-        <v>1041.11683347691</v>
+        <v>1220.66677571497</v>
       </c>
       <c r="L14" t="n">
-        <v>1102.17125446156</v>
+        <v>1292.63680251655</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B15" t="n">
-        <v>92.1189143090213</v>
+        <v>114.443058584848</v>
       </c>
       <c r="C15" t="n">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="D15" t="n">
-        <v>0.00780431430653861</v>
+        <v>0.000000898422559680867</v>
       </c>
       <c r="E15" t="n">
-        <v>0.831720001665766</v>
+        <v>0.713407573014072</v>
       </c>
       <c r="F15" t="n">
-        <v>0.788292905321447</v>
+        <v>0.629115682724094</v>
       </c>
       <c r="G15" t="n">
-        <v>0.119532045969971</v>
+        <v>0.174186719333536</v>
       </c>
       <c r="H15" t="n">
-        <v>0.0627963349733918</v>
+        <v>0.13159423009054</v>
       </c>
       <c r="I15" t="n">
-        <v>0.16857000006347</v>
+        <v>0.216937470384058</v>
       </c>
       <c r="J15" t="n">
-        <v>0.0937405583280039</v>
+        <v>0.114917901755358</v>
       </c>
       <c r="K15" t="n">
-        <v>1035.6256710619</v>
+        <v>1115.77351687684</v>
       </c>
       <c r="L15" t="n">
-        <v>1099.73281309578</v>
+        <v>1182.60282747831</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B16" t="n">
-        <v>90.9623568653841</v>
+        <v>114.72290198567</v>
       </c>
       <c r="C16" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0047577139189704</v>
+        <v>0.000000827900659250425</v>
       </c>
       <c r="E16" t="n">
-        <v>0.821420343878265</v>
+        <v>0.718437622415886</v>
       </c>
       <c r="F16" t="n">
-        <v>0.763911641059401</v>
+        <v>0.635625158420559</v>
       </c>
       <c r="G16" t="n">
-        <v>0.126227486300721</v>
+        <v>0.174570460048664</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0708421000466322</v>
+        <v>0.132012674458598</v>
       </c>
       <c r="I16" t="n">
-        <v>0.175524132563123</v>
+        <v>0.217298755875853</v>
       </c>
       <c r="J16" t="n">
-        <v>0.0908180121944795</v>
+        <v>0.111518036215793</v>
       </c>
       <c r="K16" t="n">
-        <v>1040.46911361827</v>
+        <v>1133.77920459019</v>
       </c>
       <c r="L16" t="n">
-        <v>1109.15533722599</v>
+        <v>1200.60851519166</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B17" t="n">
-        <v>181.91365249679</v>
+        <v>93.5446997268054</v>
       </c>
       <c r="C17" t="n">
-        <v>65</v>
+        <v>41</v>
       </c>
       <c r="D17" t="n">
-        <v>0.000000000000520361531641811</v>
+        <v>0.00000553465965658084</v>
       </c>
       <c r="E17" t="n">
-        <v>0.598939926186389</v>
+        <v>0.73339592976669</v>
       </c>
       <c r="F17" t="n">
-        <v>0.518727911423667</v>
+        <v>0.642360393589462</v>
       </c>
       <c r="G17" t="n">
-        <v>0.202185309739363</v>
+        <v>0.176799324170792</v>
       </c>
       <c r="H17" t="n">
-        <v>0.167739192065024</v>
+        <v>0.12954095515701</v>
       </c>
       <c r="I17" t="n">
-        <v>0.237271445976865</v>
+        <v>0.224340626631194</v>
       </c>
       <c r="J17" t="n">
-        <v>0.139320613764855</v>
+        <v>0.112415731341129</v>
       </c>
       <c r="K17" t="n">
-        <v>1267.56041596148</v>
+        <v>1029.01665984522</v>
       </c>
       <c r="L17" t="n">
-        <v>1337.14381168429</v>
+        <v>1090.70525424657</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B18" t="n">
-        <v>181.421595419391</v>
+        <v>130.476919533878</v>
       </c>
       <c r="C18" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D18" t="n">
-        <v>0.000000000000359157148466238</v>
+        <v>0.000000255995186160263</v>
       </c>
       <c r="E18" t="n">
-        <v>0.597197481042637</v>
+        <v>0.715214059714313</v>
       </c>
       <c r="F18" t="n">
-        <v>0.509084430020714</v>
+        <v>0.623503333181634</v>
       </c>
       <c r="G18" t="n">
-        <v>0.20420090532855</v>
+        <v>0.171895686777327</v>
       </c>
       <c r="H18" t="n">
-        <v>0.169574008330913</v>
+        <v>0.132111414779108</v>
       </c>
       <c r="I18" t="n">
-        <v>0.239494293393064</v>
+        <v>0.211757737314802</v>
       </c>
       <c r="J18" t="n">
-        <v>0.138890201175694</v>
+        <v>0.112319231522081</v>
       </c>
       <c r="K18" t="n">
-        <v>1269.06835888408</v>
+        <v>1220.00738793535</v>
       </c>
       <c r="L18" t="n">
-        <v>1340.43594424081</v>
+        <v>1297.11813093704</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="B19" t="n">
-        <v>116.21160703829</v>
+        <v>123.733066485582</v>
       </c>
       <c r="C19" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0000718000257309281</v>
+        <v>0.00000170961613954468</v>
       </c>
       <c r="E19" t="n">
-        <v>0.820893535309928</v>
+        <v>0.742083635852064</v>
       </c>
       <c r="F19" t="n">
-        <v>0.781713996158975</v>
+        <v>0.65902582366883</v>
       </c>
       <c r="G19" t="n">
-        <v>0.136165537621515</v>
+        <v>0.163585631964908</v>
       </c>
       <c r="H19" t="n">
-        <v>0.0958484150938124</v>
+        <v>0.123020355178999</v>
       </c>
       <c r="I19" t="n">
-        <v>0.175150416151616</v>
+        <v>0.203947621666293</v>
       </c>
       <c r="J19" t="n">
-        <v>0.111500616329999</v>
+        <v>0.116006452464026</v>
       </c>
       <c r="K19" t="n">
-        <v>1203.85837050297</v>
+        <v>1213.26353488705</v>
       </c>
       <c r="L19" t="n">
-        <v>1275.22595585971</v>
+        <v>1290.37427788875</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="B20" t="n">
-        <v>114.795113362656</v>
+        <v>125.400089023988</v>
       </c>
       <c r="C20" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0000527062409075851</v>
+        <v>0.0000101966242739282</v>
       </c>
       <c r="E20" t="n">
-        <v>0.818891877808658</v>
+        <v>0.662533424144711</v>
       </c>
       <c r="F20" t="n">
-        <v>0.772154297888312</v>
+        <v>0.595040108973653</v>
       </c>
       <c r="G20" t="n">
-        <v>0.139115230727367</v>
+        <v>0.165318955429887</v>
       </c>
       <c r="H20" t="n">
-        <v>0.098601268846195</v>
+        <v>0.121314349533521</v>
       </c>
       <c r="I20" t="n">
-        <v>0.178471063159275</v>
+        <v>0.208503860596322</v>
       </c>
       <c r="J20" t="n">
-        <v>0.111788682881206</v>
+        <v>0.105344773717229</v>
       </c>
       <c r="K20" t="n">
-        <v>1206.44187682734</v>
+        <v>1062.90684577687</v>
       </c>
       <c r="L20" t="n">
-        <v>1281.37784145191</v>
+        <v>1122.4349062369</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="B21" t="n">
-        <v>107.016917041096</v>
+        <v>115.947271574653</v>
       </c>
       <c r="C21" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D21" t="n">
-        <v>0.000132313293798036</v>
+        <v>0.0000765350681616317</v>
       </c>
       <c r="E21" t="n">
-        <v>0.835282981229819</v>
+        <v>0.709760893624499</v>
       </c>
       <c r="F21" t="n">
-        <v>0.782238517558066</v>
+        <v>0.646271089104858</v>
       </c>
       <c r="G21" t="n">
-        <v>0.136001842529632</v>
+        <v>0.154508339614438</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0939162905172976</v>
+        <v>0.108579584351779</v>
       </c>
       <c r="I21" t="n">
-        <v>0.176609650353661</v>
+        <v>0.198890851377964</v>
       </c>
       <c r="J21" t="n">
-        <v>0.110689535634113</v>
+        <v>0.100644712505223</v>
       </c>
       <c r="K21" t="n">
-        <v>1204.66368050578</v>
+        <v>1055.45402832754</v>
       </c>
       <c r="L21" t="n">
-        <v>1284.9522140321</v>
+        <v>1116.50844931218</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="B22" t="n">
-        <v>136.239614260098</v>
+        <v>101.610076724027</v>
       </c>
       <c r="C22" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D22" t="n">
-        <v>0.000000573435507189579</v>
+        <v>0.00192967430381552</v>
       </c>
       <c r="E22" t="n">
-        <v>0.733158098666727</v>
+        <v>0.789865478432134</v>
       </c>
       <c r="F22" t="n">
-        <v>0.679789718400072</v>
+        <v>0.743898551839163</v>
       </c>
       <c r="G22" t="n">
-        <v>0.159650349458825</v>
+        <v>0.131468789498287</v>
       </c>
       <c r="H22" t="n">
-        <v>0.12192162913875</v>
+        <v>0.0803594558335405</v>
       </c>
       <c r="I22" t="n">
-        <v>0.197201535433133</v>
+        <v>0.178190348491534</v>
       </c>
       <c r="J22" t="n">
-        <v>0.102376701530103</v>
+        <v>0.0968710022278117</v>
       </c>
       <c r="K22" t="n">
-        <v>1336.44750167348</v>
+        <v>1041.11683347691</v>
       </c>
       <c r="L22" t="n">
-        <v>1405.13430618553</v>
+        <v>1102.17125446156</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B23" t="n">
-        <v>117.081854913992</v>
+        <v>92.1189143090213</v>
       </c>
       <c r="C23" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D23" t="n">
-        <v>0.0000581253923876979</v>
+        <v>0.00780431430653861</v>
       </c>
       <c r="E23" t="n">
-        <v>0.801171535827923</v>
+        <v>0.831720001665766</v>
       </c>
       <c r="F23" t="n">
-        <v>0.757677809290282</v>
+        <v>0.788292905321447</v>
       </c>
       <c r="G23" t="n">
-        <v>0.138882917314024</v>
+        <v>0.119532045969971</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0982828887333949</v>
+        <v>0.0627963349733918</v>
       </c>
       <c r="I23" t="n">
-        <v>0.178221764364195</v>
+        <v>0.16857000006347</v>
       </c>
       <c r="J23" t="n">
-        <v>0.103227628896168</v>
+        <v>0.0937405583280039</v>
       </c>
       <c r="K23" t="n">
-        <v>1319.28974232738</v>
+        <v>1035.6256710619</v>
       </c>
       <c r="L23" t="n">
-        <v>1389.73774695512</v>
+        <v>1099.73281309578</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="B24" t="n">
-        <v>96.133862935031</v>
+        <v>73.2456860942102</v>
       </c>
       <c r="C24" t="n">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="D24" t="n">
-        <v>0.00577481409574587</v>
+        <v>0.0222577034934432</v>
       </c>
       <c r="E24" t="n">
-        <v>0.879636334758073</v>
+        <v>0.864754747950012</v>
       </c>
       <c r="F24" t="n">
-        <v>0.853306782986401</v>
+        <v>0.824976732641193</v>
       </c>
       <c r="G24" t="n">
-        <v>0.108058081750625</v>
+        <v>0.113265684982632</v>
       </c>
       <c r="H24" t="n">
-        <v>0.0593631424420494</v>
+        <v>0.0444795082662314</v>
       </c>
       <c r="I24" t="n">
-        <v>0.150744896758667</v>
+        <v>0.1682087923824</v>
       </c>
       <c r="J24" t="n">
-        <v>0.0875215564364808</v>
+        <v>0.0865168309568703</v>
       </c>
       <c r="K24" t="n">
-        <v>1298.34175034842</v>
+        <v>935.451130448082</v>
       </c>
       <c r="L24" t="n">
-        <v>1368.78975497616</v>
+        <v>994.979190908112</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="B25" t="n">
-        <v>77.8861593910593</v>
+        <v>70.4676896445325</v>
       </c>
       <c r="C25" t="n">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="D25" t="n">
-        <v>0.08394801559712</v>
+        <v>0.0367382904176687</v>
       </c>
       <c r="E25" t="n">
-        <v>0.940495284529242</v>
+        <v>0.872311959713835</v>
       </c>
       <c r="F25" t="n">
-        <v>0.925139228923885</v>
+        <v>0.834756653747316</v>
       </c>
       <c r="G25" t="n">
-        <v>0.0771932605317014</v>
+        <v>0.105957733637016</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>0.0278062757761363</v>
       </c>
       <c r="I25" t="n">
-        <v>0.126349261527173</v>
+        <v>0.162221026944059</v>
       </c>
       <c r="J25" t="n">
-        <v>0.082876196060517</v>
+        <v>0.104741592109844</v>
       </c>
       <c r="K25" t="n">
-        <v>1284.09404680444</v>
+        <v>981.557952855311</v>
       </c>
       <c r="L25" t="n">
-        <v>1358.06445166357</v>
+        <v>1041.08601331534</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="B26" t="n">
-        <v>74.6593477129279</v>
+        <v>53.2799068039664</v>
       </c>
       <c r="C26" t="n">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="D26" t="n">
-        <v>0.082127828305905</v>
+        <v>0.0946989536156793</v>
       </c>
       <c r="E26" t="n">
-        <v>0.941344852007474</v>
+        <v>0.910346825137198</v>
       </c>
       <c r="F26" t="n">
-        <v>0.922455906043779</v>
+        <v>0.879733545915754</v>
       </c>
       <c r="G26" t="n">
-        <v>0.0785645450984261</v>
+        <v>0.0938568876234015</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
       </c>
       <c r="I26" t="n">
+        <v>0.159037545073325</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.093144197325303</v>
+      </c>
+      <c r="K26" t="n">
+        <v>883.063613015609</v>
+      </c>
+      <c r="L26" t="n">
+        <v>938.012591901791</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" t="n">
+        <v>90.9623568653841</v>
+      </c>
+      <c r="C27" t="n">
+        <v>59</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.0047577139189704</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.821420343878265</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.763911641059401</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.126227486300721</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.0708421000466322</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.175524132563123</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.0908180121944795</v>
+      </c>
+      <c r="K27" t="n">
+        <v>1040.46911361827</v>
+      </c>
+      <c r="L27" t="n">
+        <v>1109.15533722599</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" t="n">
+        <v>93.9450110436006</v>
+      </c>
+      <c r="C28" t="n">
+        <v>59</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.00257555253269615</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.804755698035054</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.741880414351427</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.131985774943507</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.0786856937622018</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.180547694096942</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.0941772495193381</v>
+      </c>
+      <c r="K28" t="n">
+        <v>1043.45176779648</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1112.13799140421</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" t="n">
+        <v>181.91365249679</v>
+      </c>
+      <c r="C29" t="n">
+        <v>65</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.000000000000520361531641811</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.598939926186389</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.518727911423667</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.202185309739363</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.167739192065024</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.237271445976865</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.139320613764855</v>
+      </c>
+      <c r="K29" t="n">
+        <v>1267.56041596148</v>
+      </c>
+      <c r="L29" t="n">
+        <v>1337.14381168429</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" t="n">
+        <v>181.421595419391</v>
+      </c>
+      <c r="C30" t="n">
+        <v>64</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.000000000000359157148466238</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.597197481042637</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.509084430020714</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.20420090532855</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.169574008330913</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.239494293393064</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.138890201175694</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1269.06835888408</v>
+      </c>
+      <c r="L30" t="n">
+        <v>1340.43594424081</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" t="n">
+        <v>116.21160703829</v>
+      </c>
+      <c r="C31" t="n">
+        <v>64</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.0000718000257309281</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.820893535309928</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.781713996158975</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.136165537621515</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.0958484150938124</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.175150416151616</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.111500616329999</v>
+      </c>
+      <c r="K31" t="n">
+        <v>1203.85837050297</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1275.22595585971</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>60</v>
+      </c>
+      <c r="B32" t="n">
+        <v>114.795113362656</v>
+      </c>
+      <c r="C32" t="n">
+        <v>62</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.0000527062409075851</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.818891877808658</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.772154297888312</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.139115230727367</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.098601268846195</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.178471063159275</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.111788682881206</v>
+      </c>
+      <c r="K32" t="n">
+        <v>1206.44187682734</v>
+      </c>
+      <c r="L32" t="n">
+        <v>1281.37784145191</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" t="n">
+        <v>95.6656313141923</v>
+      </c>
+      <c r="C33" t="n">
+        <v>51</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.00015324971982722</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.824882382811145</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.773377201285011</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.141083203403583</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.0965971337562586</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.184283958585547</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.117934015081639</v>
+      </c>
+      <c r="K33" t="n">
+        <v>1115.22354895608</v>
+      </c>
+      <c r="L33" t="n">
+        <v>1184.80694467889</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>62</v>
+      </c>
+      <c r="B34" t="n">
+        <v>97.1180628013245</v>
+      </c>
+      <c r="C34" t="n">
+        <v>51</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.000105793458435866</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.82682497790973</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.775891147883179</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.143358715783047</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.0992481312377277</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.186365986564836</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.111477202179966</v>
+      </c>
+      <c r="K34" t="n">
+        <v>1117.52416020274</v>
+      </c>
+      <c r="L34" t="n">
+        <v>1187.10755592555</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>63</v>
+      </c>
+      <c r="B35" t="n">
+        <v>83.2994984989401</v>
+      </c>
+      <c r="C35" t="n">
+        <v>41</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.000104900908168726</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.816852789463734</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.754314717573301</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.153126142692583</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.105373897382169</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.200249460024962</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.119299308332113</v>
+      </c>
+      <c r="K35" t="n">
+        <v>1029.51589697444</v>
+      </c>
+      <c r="L35" t="n">
+        <v>1093.7467237955</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>64</v>
+      </c>
+      <c r="B36" t="n">
+        <v>107.016917041096</v>
+      </c>
+      <c r="C36" t="n">
+        <v>59</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.000132313293798036</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.835282981229819</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.782238517558066</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.136001842529632</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.0939162905172976</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.176609650353661</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.110689535634113</v>
+      </c>
+      <c r="K36" t="n">
+        <v>1204.66368050578</v>
+      </c>
+      <c r="L36" t="n">
+        <v>1284.9522140321</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>65</v>
+      </c>
+      <c r="B37" t="n">
+        <v>110.799663829104</v>
+      </c>
+      <c r="C37" t="n">
+        <v>59</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.0000519563700150938</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.822306663463523</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.765083385595844</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.141257373410376</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.100024874788608</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.181419421020551</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.111947428125996</v>
+      </c>
+      <c r="K37" t="n">
+        <v>1208.44642729379</v>
+      </c>
+      <c r="L37" t="n">
+        <v>1288.73496082011</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>66</v>
+      </c>
+      <c r="B38" t="n">
+        <v>136.239614260098</v>
+      </c>
+      <c r="C38" t="n">
+        <v>65</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.000000573435507189579</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.733158098666727</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.679789718400072</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.159650349458825</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.12192162913875</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.197201535433133</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.102376701530103</v>
+      </c>
+      <c r="K38" t="n">
+        <v>1336.44750167348</v>
+      </c>
+      <c r="L38" t="n">
+        <v>1405.13430618553</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>67</v>
+      </c>
+      <c r="B39" t="n">
+        <v>117.081854913992</v>
+      </c>
+      <c r="C39" t="n">
+        <v>64</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.0000581253923876979</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.801171535827923</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.757677809290282</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.138882917314024</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.0982828887333949</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.178221764364195</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.103227628896168</v>
+      </c>
+      <c r="K39" t="n">
+        <v>1319.28974232738</v>
+      </c>
+      <c r="L39" t="n">
+        <v>1389.73774695512</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>68</v>
+      </c>
+      <c r="B40" t="n">
+        <v>96.133862935031</v>
+      </c>
+      <c r="C40" t="n">
+        <v>64</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.00577481409574587</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.879636334758073</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.853306782986401</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.108058081750625</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.0593631424420494</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.150744896758667</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0.0875215564364808</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1298.34175034842</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1368.78975497616</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>69</v>
+      </c>
+      <c r="B41" t="n">
+        <v>77.8861593910593</v>
+      </c>
+      <c r="C41" t="n">
+        <v>62</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.08394801559712</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.940495284529242</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.925139228923885</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.0771932605317014</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.126349261527173</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.082876196060517</v>
+      </c>
+      <c r="K41" t="n">
+        <v>1284.09404680444</v>
+      </c>
+      <c r="L41" t="n">
+        <v>1358.06445166357</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" t="n">
+        <v>62.2430765088063</v>
+      </c>
+      <c r="C42" t="n">
+        <v>51</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.134471186505739</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.955358956932874</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.94222923838372</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.071601689041535</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.126974071893411</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0.0839664175297392</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1176.70729771637</v>
+      </c>
+      <c r="L42" t="n">
+        <v>1245.39410222842</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>71</v>
+      </c>
+      <c r="B43" t="n">
+        <v>57.7565711154923</v>
+      </c>
+      <c r="C43" t="n">
+        <v>51</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.239807395647922</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.971079113116618</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.962572969915623</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.0555065021496604</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.116303057373456</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.0782665541101585</v>
+      </c>
+      <c r="K43" t="n">
+        <v>1193.43242845741</v>
+      </c>
+      <c r="L43" t="n">
+        <v>1262.11923296946</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>72</v>
+      </c>
+      <c r="B44" t="n">
+        <v>42.408847525499</v>
+      </c>
+      <c r="C44" t="n">
+        <v>41</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.410082784292924</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.993532215172617</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.99132370328034</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.0282687002392316</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.109424102051244</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.0781845679029616</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1086.0202564973</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1149.42346066227</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>73</v>
+      </c>
+      <c r="B45" t="n">
+        <v>74.6593477129279</v>
+      </c>
+      <c r="C45" t="n">
+        <v>59</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0.082127828305905</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.941344852007474</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.922455906043779</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.0785645450984261</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="n">
         <v>0.12853159284671</v>
       </c>
-      <c r="J26" t="n">
+      <c r="J45" t="n">
         <v>0.0788285311350711</v>
       </c>
-      <c r="K26" t="n">
+      <c r="K45" t="n">
         <v>1286.86723512631</v>
       </c>
-      <c r="L26" t="n">
+      <c r="L45" t="n">
         <v>1366.12124033252</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>74</v>
+      </c>
+      <c r="B46" t="n">
+        <v>77.7611408624681</v>
+      </c>
+      <c r="C46" t="n">
+        <v>59</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.0513527699485115</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.929726479418539</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.907096023638069</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.0859942451220681</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0.13426940115362</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0.0827713059191711</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1289.96902827585</v>
+      </c>
+      <c r="L46" t="n">
+        <v>1369.22303348206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>